<commit_message>
refactor to app-specific slide levels
</commit_message>
<xml_diff>
--- a/app-outline.xlsx
+++ b/app-outline.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilsonte\University of Michigan Dropbox\Thomas Wilson\WILSONTE_DROPBOX\um-agentic-ed\um-agentic-ed-docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9EB472A-3636-432B-8561-9FE478211AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F0EBABC-8FB3-46C6-A720-60328AE898DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16590" yWindow="0" windowWidth="12315" windowHeight="17385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4395" yWindow="1050" windowWidth="23580" windowHeight="13830" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="87">
   <si>
     <t>Subject</t>
   </si>
@@ -51,12 +51,6 @@
     <t>AI-Generated Content</t>
   </si>
   <si>
-    <t>Obtaining an App</t>
-  </si>
-  <si>
-    <t>App Distibution Types</t>
-  </si>
-  <si>
     <t>Navigating through slides</t>
   </si>
   <si>
@@ -162,12 +156,6 @@
     <t>Using an Agent</t>
   </si>
   <si>
-    <t>Clone  an app repository</t>
-  </si>
-  <si>
-    <t>Opening an app in your web browser</t>
-  </si>
-  <si>
     <t>Learner Mode</t>
   </si>
   <si>
@@ -177,15 +165,9 @@
     <t>Basic UI Usage</t>
   </si>
   <si>
-    <t>Hiding the sidebar</t>
-  </si>
-  <si>
     <t>Searching for text keywords</t>
   </si>
   <si>
-    <t>Using the sidebar</t>
-  </si>
-  <si>
     <t>Interactive slide widgets</t>
   </si>
   <si>
@@ -201,21 +183,12 @@
     <t>Interactive Slide Features</t>
   </si>
   <si>
-    <t>Note Taking</t>
-  </si>
-  <si>
     <t>Data file upload</t>
   </si>
   <si>
-    <t>Entering  presenter mode</t>
-  </si>
-  <si>
     <t>Changing slide text size</t>
   </si>
   <si>
-    <t>Single exported app HTML files</t>
-  </si>
-  <si>
     <t>Taking text notes</t>
   </si>
   <si>
@@ -231,9 +204,6 @@
     <t>Using widgets while presenting</t>
   </si>
   <si>
-    <t>Live presenter features</t>
-  </si>
-  <si>
     <t>Verify the installation in a web browser</t>
   </si>
   <si>
@@ -298,6 +268,24 @@
   </si>
   <si>
     <t>Using agent skill `migrate-app`</t>
+  </si>
+  <si>
+    <t>Using the header and sidebar</t>
+  </si>
+  <si>
+    <t>Navigating through a section's slides</t>
+  </si>
+  <si>
+    <t>Entering  and exiting presenter mode</t>
+  </si>
+  <si>
+    <t>Accessing an App</t>
+  </si>
+  <si>
+    <t>Live Presenter Features</t>
+  </si>
+  <si>
+    <t>Note Taking and Sketches</t>
   </si>
 </sst>
 </file>
@@ -624,7 +612,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -648,24 +636,24 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -673,231 +661,231 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D15" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D16" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C17" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="D17" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E17" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E19" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D20" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="E20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D21" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="E21" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D22" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E23" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D24" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="E24" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D25" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D26" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E26" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D27" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E27" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.25">
@@ -905,193 +893,193 @@
         <v>7</v>
       </c>
       <c r="D29" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E29" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D30" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E30" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D31" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D32" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E32" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C33" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D33" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="E33" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E34" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="C35" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D35" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E35" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D36" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E36" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D37" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C38" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D38" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
       <c r="D39" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E39" t="s">
-        <v>15</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>43</v>
+      </c>
+      <c r="C40" t="s">
+        <v>45</v>
+      </c>
       <c r="D40" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="E40" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C41" t="s">
-        <v>4</v>
-      </c>
       <c r="D41" t="s">
+        <v>82</v>
+      </c>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D42" t="s">
         <v>46</v>
       </c>
-      <c r="E41" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B42" t="s">
+      <c r="E42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C43" t="s">
+        <v>51</v>
+      </c>
+      <c r="D43" t="s">
         <v>47</v>
       </c>
-      <c r="C42" t="s">
-        <v>49</v>
-      </c>
-      <c r="D42" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D43" t="s">
-        <v>52</v>
-      </c>
       <c r="E43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D44" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="D45" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C46" t="s">
-        <v>57</v>
-      </c>
       <c r="D46" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E46" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C47" t="s">
+        <v>86</v>
+      </c>
       <c r="D47" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="E47" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1099,99 +1087,72 @@
         <v>55</v>
       </c>
       <c r="E48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D49" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C50" t="s">
-        <v>58</v>
-      </c>
       <c r="D50" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51" t="s">
+        <v>44</v>
+      </c>
+      <c r="C51" t="s">
+        <v>45</v>
+      </c>
       <c r="D51" t="s">
-        <v>64</v>
+        <v>83</v>
       </c>
       <c r="E51" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D52" t="s">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="E52" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D53" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E53" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B54" t="s">
-        <v>48</v>
-      </c>
       <c r="C54" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="D54" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D55" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
       <c r="E55" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D56" t="s">
-        <v>61</v>
-      </c>
-      <c r="E56" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="C57" t="s">
-        <v>68</v>
-      </c>
-      <c r="D57" t="s">
-        <v>66</v>
-      </c>
-      <c r="E57" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="D58" t="s">
-        <v>67</v>
-      </c>
-      <c r="E58" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>